<commit_message>
Atualização dos arquivos Excel
</commit_message>
<xml_diff>
--- a/crm_dominus/apps/dados/backlog_adesao.xlsx
+++ b/crm_dominus/apps/dados/backlog_adesao.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PME-COM-02740\Desktop\CRM_Dominus\crm_dominus\apps\dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PME-COM-02740\Desktop\V2-crm-dominus\crm_dominus\apps\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4BEF108-AF62-486E-9229-CFBB1E6468D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B6ECAA-76D9-4A38-B71D-E2C766978517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F9C4030F-1739-402F-A3F2-D33CA6562C8E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4632" uniqueCount="1068">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4634" uniqueCount="1069">
   <si>
     <t>Cliente</t>
   </si>
@@ -3238,6 +3238,9 @@
   </si>
   <si>
     <t>O&amp;M - GRP - FERNANDO SZCZEREPA CASSOL</t>
+  </si>
+  <si>
+    <t>PAR - TER - GTI - M.A MARTINS TELECOM LTDA</t>
   </si>
 </sst>
 </file>
@@ -20612,11 +20615,11 @@
       <c r="D652" s="7">
         <v>873883</v>
       </c>
-      <c r="E652" s="5">
-        <v>0</v>
-      </c>
-      <c r="F652" s="5">
-        <v>0</v>
+      <c r="E652" s="5" t="s">
+        <v>1068</v>
+      </c>
+      <c r="F652" s="5" t="s">
+        <v>255</v>
       </c>
       <c r="G652" s="5" t="s">
         <v>199</v>

</xml_diff>